<commit_message>
Latest Files Or BOM  LCSC or Digikey
</commit_message>
<xml_diff>
--- a/Deliverables/Core-Production-Files/BOM/BOM_Digikey.xlsx
+++ b/Deliverables/Core-Production-Files/BOM/BOM_Digikey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faiza\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\MatrixProject-JohnWollam\Deliverables\Core-Production-Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="259">
   <si>
     <t>S. No.</t>
   </si>
@@ -794,6 +794,15 @@
   </si>
   <si>
     <t>R1, R4, R59, R60, R61, R62, R63, R64, R65, R66, R71, R72, R73, R74, R75, R76, R77, R78, R83, R84, R85, R86, R90, R91, R92, R93, R94, R95, R96, R97, R102, R103, R104, R105, R106, R107, R108, R109, R114, R115, R116, R117, R120, R121, R122, R123, R12, R19, R20, R25, R26, RF3</t>
+  </si>
+  <si>
+    <t>Unit Cost (110 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (110)</t>
+  </si>
+  <si>
+    <t>Quantity 110</t>
   </si>
 </sst>
 </file>
@@ -945,7 +954,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -1408,12 +1417,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1716,19 +1751,83 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1737,69 +1836,11 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="37" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2082,7 +2123,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q56"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -2096,36 +2137,42 @@
     <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="32.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="120" t="s">
+    <row r="1" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="129" t="s">
         <v>252</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-    </row>
-    <row r="2" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="130"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="130"/>
+      <c r="L1" s="130"/>
+      <c r="M1" s="130"/>
+      <c r="N1" s="130"/>
+      <c r="O1" s="130"/>
+      <c r="P1" s="130"/>
+      <c r="Q1" s="130"/>
+      <c r="R1" s="130"/>
+      <c r="S1" s="130"/>
+      <c r="T1" s="130"/>
+    </row>
+    <row r="2" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2159,30 +2206,39 @@
       <c r="K2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="T2" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="117" t="s">
+      <c r="B3" s="134" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="6" t="s">
@@ -2213,30 +2269,41 @@
         <f>J3*80*1.1</f>
         <v>352</v>
       </c>
-      <c r="L3" s="41" t="s">
+      <c r="L3" s="8">
+        <f>J3*110</f>
+        <v>440</v>
+      </c>
+      <c r="M3" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="M3" s="55">
+      <c r="N3" s="55">
         <v>0.37</v>
       </c>
-      <c r="N3" s="10">
-        <f>M3*J3</f>
+      <c r="O3" s="10">
+        <f>N3*J3</f>
         <v>1.48</v>
       </c>
-      <c r="O3" s="55">
+      <c r="P3" s="55">
         <v>0.15479999999999999</v>
       </c>
-      <c r="P3" s="10">
-        <f>O3*K3</f>
+      <c r="Q3" s="10">
+        <f>P3*K3</f>
         <v>54.489599999999996</v>
       </c>
-      <c r="Q3" s="11"/>
-    </row>
-    <row r="4" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R3" s="55">
+        <v>0.15479999999999999</v>
+      </c>
+      <c r="S3" s="139">
+        <f>R3*L3</f>
+        <v>68.111999999999995</v>
+      </c>
+      <c r="T3" s="11"/>
+    </row>
+    <row r="4" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="118"/>
+      <c r="B4" s="135"/>
       <c r="C4" s="12" t="s">
         <v>30</v>
       </c>
@@ -2265,30 +2332,41 @@
         <f>J4*80*1.1</f>
         <v>88</v>
       </c>
-      <c r="L4" s="39" t="s">
+      <c r="L4" s="8">
+        <f t="shared" ref="L4:L49" si="0">J4*110</f>
+        <v>110</v>
+      </c>
+      <c r="M4" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="M4" s="56">
+      <c r="N4" s="56">
         <v>1.69</v>
       </c>
-      <c r="N4" s="50">
-        <f t="shared" ref="N4:N48" si="0">M4*J4</f>
+      <c r="O4" s="50">
+        <f t="shared" ref="O4:O48" si="1">N4*J4</f>
         <v>1.69</v>
       </c>
-      <c r="O4" s="56">
+      <c r="P4" s="56">
         <v>1.1566000000000001</v>
       </c>
-      <c r="P4" s="50">
-        <f t="shared" ref="P4:P48" si="1">O4*K4</f>
+      <c r="Q4" s="50">
+        <f t="shared" ref="Q4:Q48" si="2">P4*K4</f>
         <v>101.7808</v>
       </c>
-      <c r="Q4" s="17"/>
-    </row>
-    <row r="5" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R4" s="56">
+        <v>1.1566000000000001</v>
+      </c>
+      <c r="S4" s="139">
+        <f t="shared" ref="S4:S48" si="3">R4*L4</f>
+        <v>127.22600000000001</v>
+      </c>
+      <c r="T4" s="17"/>
+    </row>
+    <row r="5" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="118"/>
+      <c r="B5" s="135"/>
       <c r="C5" s="12" t="s">
         <v>35</v>
       </c>
@@ -2314,33 +2392,44 @@
         <v>1</v>
       </c>
       <c r="K5" s="16">
-        <f t="shared" ref="K5:K15" si="2">J5*80*1.1</f>
+        <f t="shared" ref="K5:K15" si="4">J5*80*1.1</f>
         <v>88</v>
       </c>
-      <c r="L5" s="39" t="s">
+      <c r="L5" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M5" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="M5" s="56">
+      <c r="N5" s="56">
         <v>0.54</v>
       </c>
-      <c r="N5" s="50">
-        <f t="shared" si="0"/>
+      <c r="O5" s="50">
+        <f t="shared" si="1"/>
         <v>0.54</v>
       </c>
-      <c r="O5" s="56">
+      <c r="P5" s="56">
         <v>0.28820000000000001</v>
       </c>
-      <c r="P5" s="50">
-        <f t="shared" si="1"/>
+      <c r="Q5" s="50">
+        <f t="shared" si="2"/>
         <v>25.361600000000003</v>
       </c>
-      <c r="Q5" s="17"/>
-    </row>
-    <row r="6" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R5" s="56">
+        <v>0.28820000000000001</v>
+      </c>
+      <c r="S5" s="139">
+        <f t="shared" si="3"/>
+        <v>31.702000000000002</v>
+      </c>
+      <c r="T5" s="17"/>
+    </row>
+    <row r="6" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="118"/>
+      <c r="B6" s="135"/>
       <c r="C6" s="12" t="s">
         <v>39</v>
       </c>
@@ -2366,33 +2455,44 @@
         <v>1</v>
       </c>
       <c r="K6" s="16">
+        <f t="shared" si="4"/>
+        <v>88</v>
+      </c>
+      <c r="L6" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M6" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N6" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O6" s="50">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="P6" s="56">
+        <v>3.7199999999999997E-2</v>
+      </c>
+      <c r="Q6" s="50">
         <f t="shared" si="2"/>
-        <v>88</v>
-      </c>
-      <c r="L6" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M6" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N6" s="50">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-      <c r="O6" s="56">
+        <v>3.2735999999999996</v>
+      </c>
+      <c r="R6" s="56">
         <v>3.7199999999999997E-2</v>
       </c>
-      <c r="P6" s="50">
-        <f t="shared" si="1"/>
-        <v>3.2735999999999996</v>
-      </c>
-      <c r="Q6" s="17"/>
-    </row>
-    <row r="7" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S6" s="139">
+        <f t="shared" si="3"/>
+        <v>4.0919999999999996</v>
+      </c>
+      <c r="T6" s="17"/>
+    </row>
+    <row r="7" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="118"/>
+      <c r="B7" s="135"/>
       <c r="C7" s="12" t="s">
         <v>44</v>
       </c>
@@ -2418,33 +2518,44 @@
         <v>2</v>
       </c>
       <c r="K7" s="16">
+        <f t="shared" si="4"/>
+        <v>176</v>
+      </c>
+      <c r="L7" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M7" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N7" s="56">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="O7" s="50">
+        <f t="shared" si="1"/>
+        <v>2.1800000000000002</v>
+      </c>
+      <c r="P7" s="56">
+        <v>0.64690000000000003</v>
+      </c>
+      <c r="Q7" s="50">
         <f t="shared" si="2"/>
-        <v>176</v>
-      </c>
-      <c r="L7" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M7" s="56">
-        <v>1.0900000000000001</v>
-      </c>
-      <c r="N7" s="50">
-        <f t="shared" si="0"/>
-        <v>2.1800000000000002</v>
-      </c>
-      <c r="O7" s="56">
+        <v>113.8544</v>
+      </c>
+      <c r="R7" s="56">
         <v>0.64690000000000003</v>
       </c>
-      <c r="P7" s="50">
-        <f t="shared" si="1"/>
-        <v>113.8544</v>
-      </c>
-      <c r="Q7" s="17"/>
-    </row>
-    <row r="8" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S7" s="139">
+        <f t="shared" si="3"/>
+        <v>142.31800000000001</v>
+      </c>
+      <c r="T7" s="17"/>
+    </row>
+    <row r="8" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="118"/>
+      <c r="B8" s="135"/>
       <c r="C8" s="12" t="s">
         <v>49</v>
       </c>
@@ -2470,33 +2581,44 @@
         <v>2</v>
       </c>
       <c r="K8" s="16">
+        <f t="shared" si="4"/>
+        <v>176</v>
+      </c>
+      <c r="L8" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M8" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N8" s="56">
+        <v>0.38</v>
+      </c>
+      <c r="O8" s="50">
+        <f t="shared" si="1"/>
+        <v>0.76</v>
+      </c>
+      <c r="P8" s="56">
+        <v>0.1474</v>
+      </c>
+      <c r="Q8" s="50">
         <f t="shared" si="2"/>
-        <v>176</v>
-      </c>
-      <c r="L8" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M8" s="56">
-        <v>0.38</v>
-      </c>
-      <c r="N8" s="50">
-        <f t="shared" si="0"/>
-        <v>0.76</v>
-      </c>
-      <c r="O8" s="56">
+        <v>25.942399999999999</v>
+      </c>
+      <c r="R8" s="56">
         <v>0.1474</v>
       </c>
-      <c r="P8" s="50">
-        <f t="shared" si="1"/>
-        <v>25.942399999999999</v>
-      </c>
-      <c r="Q8" s="17"/>
-    </row>
-    <row r="9" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S8" s="139">
+        <f t="shared" si="3"/>
+        <v>32.427999999999997</v>
+      </c>
+      <c r="T8" s="17"/>
+    </row>
+    <row r="9" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="118"/>
+      <c r="B9" s="135"/>
       <c r="C9" s="12" t="s">
         <v>54</v>
       </c>
@@ -2522,33 +2644,44 @@
         <v>2</v>
       </c>
       <c r="K9" s="16">
+        <f t="shared" si="4"/>
+        <v>176</v>
+      </c>
+      <c r="L9" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M9" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N9" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="O9" s="50">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="P9" s="56">
+        <v>0.23219999999999999</v>
+      </c>
+      <c r="Q9" s="50">
         <f t="shared" si="2"/>
-        <v>176</v>
-      </c>
-      <c r="L9" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M9" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="N9" s="50">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="O9" s="56">
+        <v>40.867199999999997</v>
+      </c>
+      <c r="R9" s="56">
         <v>0.23219999999999999</v>
       </c>
-      <c r="P9" s="50">
-        <f t="shared" si="1"/>
-        <v>40.867199999999997</v>
-      </c>
-      <c r="Q9" s="17"/>
-    </row>
-    <row r="10" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S9" s="139">
+        <f t="shared" si="3"/>
+        <v>51.083999999999996</v>
+      </c>
+      <c r="T9" s="17"/>
+    </row>
+    <row r="10" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="118"/>
+      <c r="B10" s="135"/>
       <c r="C10" s="12" t="s">
         <v>58</v>
       </c>
@@ -2574,33 +2707,44 @@
         <v>2</v>
       </c>
       <c r="K10" s="16">
+        <f t="shared" si="4"/>
+        <v>176</v>
+      </c>
+      <c r="L10" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M10" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N10" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="O10" s="50">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="P10" s="56">
+        <v>0.23469999999999999</v>
+      </c>
+      <c r="Q10" s="50">
         <f t="shared" si="2"/>
-        <v>176</v>
-      </c>
-      <c r="L10" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M10" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="N10" s="50">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="O10" s="56">
+        <v>41.307200000000002</v>
+      </c>
+      <c r="R10" s="56">
         <v>0.23469999999999999</v>
       </c>
-      <c r="P10" s="50">
-        <f t="shared" si="1"/>
-        <v>41.307200000000002</v>
-      </c>
-      <c r="Q10" s="17"/>
-    </row>
-    <row r="11" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S10" s="139">
+        <f t="shared" si="3"/>
+        <v>51.634</v>
+      </c>
+      <c r="T10" s="17"/>
+    </row>
+    <row r="11" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="118"/>
+      <c r="B11" s="135"/>
       <c r="C11" s="12" t="s">
         <v>26</v>
       </c>
@@ -2626,33 +2770,44 @@
         <v>4</v>
       </c>
       <c r="K11" s="16">
+        <f t="shared" si="4"/>
+        <v>352</v>
+      </c>
+      <c r="L11" s="8">
+        <f t="shared" si="0"/>
+        <v>440</v>
+      </c>
+      <c r="M11" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N11" s="56">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="O11" s="50">
+        <f t="shared" si="1"/>
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="P11" s="56">
+        <v>0.26919999999999999</v>
+      </c>
+      <c r="Q11" s="50">
         <f t="shared" si="2"/>
-        <v>352</v>
-      </c>
-      <c r="L11" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M11" s="56">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="N11" s="50">
-        <f t="shared" si="0"/>
-        <v>2.3199999999999998</v>
-      </c>
-      <c r="O11" s="56">
+        <v>94.758399999999995</v>
+      </c>
+      <c r="R11" s="56">
         <v>0.26919999999999999</v>
       </c>
-      <c r="P11" s="50">
-        <f t="shared" si="1"/>
-        <v>94.758399999999995</v>
-      </c>
-      <c r="Q11" s="17"/>
-    </row>
-    <row r="12" spans="1:17" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S11" s="139">
+        <f t="shared" si="3"/>
+        <v>118.44799999999999</v>
+      </c>
+      <c r="T11" s="17"/>
+    </row>
+    <row r="12" spans="1:20" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="118"/>
+      <c r="B12" s="135"/>
       <c r="C12" s="76" t="s">
         <v>63</v>
       </c>
@@ -2678,33 +2833,44 @@
         <v>14</v>
       </c>
       <c r="K12" s="16">
+        <f t="shared" si="4"/>
+        <v>1232</v>
+      </c>
+      <c r="L12" s="8">
+        <f t="shared" si="0"/>
+        <v>1540</v>
+      </c>
+      <c r="M12" s="72" t="s">
+        <v>225</v>
+      </c>
+      <c r="N12" s="73">
+        <v>0.03</v>
+      </c>
+      <c r="O12" s="74">
+        <f t="shared" si="1"/>
+        <v>0.42</v>
+      </c>
+      <c r="P12" s="73">
+        <v>7.5900000000000004E-3</v>
+      </c>
+      <c r="Q12" s="74">
         <f t="shared" si="2"/>
-        <v>1232</v>
-      </c>
-      <c r="L12" s="72" t="s">
-        <v>225</v>
-      </c>
-      <c r="M12" s="73">
-        <v>0.03</v>
-      </c>
-      <c r="N12" s="74">
-        <f t="shared" si="0"/>
-        <v>0.42</v>
-      </c>
-      <c r="O12" s="73">
+        <v>9.3508800000000001</v>
+      </c>
+      <c r="R12" s="73">
         <v>7.5900000000000004E-3</v>
       </c>
-      <c r="P12" s="74">
-        <f t="shared" si="1"/>
-        <v>9.3508800000000001</v>
-      </c>
-      <c r="Q12" s="75"/>
-    </row>
-    <row r="13" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S12" s="139">
+        <f t="shared" si="3"/>
+        <v>11.688600000000001</v>
+      </c>
+      <c r="T12" s="75"/>
+    </row>
+    <row r="13" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="118"/>
+      <c r="B13" s="135"/>
       <c r="C13" s="12" t="s">
         <v>65</v>
       </c>
@@ -2730,33 +2896,44 @@
         <v>1</v>
       </c>
       <c r="K13" s="16">
+        <f t="shared" si="4"/>
+        <v>88</v>
+      </c>
+      <c r="L13" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M13" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N13" s="56">
+        <v>0.3</v>
+      </c>
+      <c r="O13" s="50">
+        <f t="shared" si="1"/>
+        <v>0.3</v>
+      </c>
+      <c r="P13" s="56">
+        <v>0.1236</v>
+      </c>
+      <c r="Q13" s="50">
         <f t="shared" si="2"/>
-        <v>88</v>
-      </c>
-      <c r="L13" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M13" s="56">
-        <v>0.3</v>
-      </c>
-      <c r="N13" s="50">
-        <f t="shared" si="0"/>
-        <v>0.3</v>
-      </c>
-      <c r="O13" s="56">
+        <v>10.876799999999999</v>
+      </c>
+      <c r="R13" s="56">
         <v>0.1236</v>
       </c>
-      <c r="P13" s="50">
-        <f t="shared" si="1"/>
-        <v>10.876799999999999</v>
-      </c>
-      <c r="Q13" s="17"/>
-    </row>
-    <row r="14" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S13" s="139">
+        <f t="shared" si="3"/>
+        <v>13.596</v>
+      </c>
+      <c r="T13" s="17"/>
+    </row>
+    <row r="14" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="118"/>
+      <c r="B14" s="135"/>
       <c r="C14" s="12" t="s">
         <v>69</v>
       </c>
@@ -2780,33 +2957,44 @@
         <v>1</v>
       </c>
       <c r="K14" s="16">
+        <f t="shared" si="4"/>
+        <v>88</v>
+      </c>
+      <c r="L14" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M14" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N14" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O14" s="50">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="P14" s="56">
+        <v>1.0200000000000001E-2</v>
+      </c>
+      <c r="Q14" s="50">
         <f t="shared" si="2"/>
-        <v>88</v>
-      </c>
-      <c r="L14" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M14" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N14" s="50">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-      <c r="O14" s="56">
+        <v>0.89760000000000006</v>
+      </c>
+      <c r="R14" s="56">
         <v>1.0200000000000001E-2</v>
       </c>
-      <c r="P14" s="50">
-        <f t="shared" si="1"/>
-        <v>0.89760000000000006</v>
-      </c>
-      <c r="Q14" s="17"/>
-    </row>
-    <row r="15" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S14" s="139">
+        <f t="shared" si="3"/>
+        <v>1.1220000000000001</v>
+      </c>
+      <c r="T14" s="17"/>
+    </row>
+    <row r="15" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="119"/>
+      <c r="B15" s="136"/>
       <c r="C15" s="19" t="s">
         <v>73</v>
       </c>
@@ -2832,33 +3020,44 @@
         <v>2</v>
       </c>
       <c r="K15" s="16">
+        <f t="shared" si="4"/>
+        <v>176</v>
+      </c>
+      <c r="L15" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M15" s="40" t="s">
+        <v>225</v>
+      </c>
+      <c r="N15" s="57">
+        <v>0.1</v>
+      </c>
+      <c r="O15" s="51">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="P15" s="57">
+        <v>1.2200000000000001E-2</v>
+      </c>
+      <c r="Q15" s="51">
         <f t="shared" si="2"/>
-        <v>176</v>
-      </c>
-      <c r="L15" s="40" t="s">
-        <v>225</v>
-      </c>
-      <c r="M15" s="57">
-        <v>0.1</v>
-      </c>
-      <c r="N15" s="51">
-        <f t="shared" si="0"/>
-        <v>0.2</v>
-      </c>
-      <c r="O15" s="57">
+        <v>2.1472000000000002</v>
+      </c>
+      <c r="R15" s="57">
         <v>1.2200000000000001E-2</v>
       </c>
-      <c r="P15" s="51">
-        <f t="shared" si="1"/>
-        <v>2.1472000000000002</v>
-      </c>
-      <c r="Q15" s="23"/>
-    </row>
-    <row r="16" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S15" s="139">
+        <f t="shared" si="3"/>
+        <v>2.6840000000000002</v>
+      </c>
+      <c r="T15" s="23"/>
+    </row>
+    <row r="16" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="113" t="s">
+      <c r="B16" s="131" t="s">
         <v>77</v>
       </c>
       <c r="C16" s="6" t="s">
@@ -2886,33 +3085,44 @@
         <v>2</v>
       </c>
       <c r="K16" s="8">
-        <f>J16*80*1.1</f>
+        <f t="shared" ref="K16:K28" si="5">J16*80*1.1</f>
         <v>176</v>
       </c>
-      <c r="L16" s="41" t="s">
+      <c r="L16" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M16" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="M16" s="55">
+      <c r="N16" s="55">
         <v>0.42</v>
       </c>
-      <c r="N16" s="52">
-        <f t="shared" si="0"/>
+      <c r="O16" s="52">
+        <f t="shared" si="1"/>
         <v>0.84</v>
       </c>
-      <c r="O16" s="55">
+      <c r="P16" s="55">
         <v>0.1948</v>
       </c>
-      <c r="P16" s="52">
-        <f t="shared" si="1"/>
+      <c r="Q16" s="52">
+        <f t="shared" si="2"/>
         <v>34.284799999999997</v>
       </c>
-      <c r="Q16" s="11"/>
-    </row>
-    <row r="17" spans="1:17" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R16" s="55">
+        <v>0.1948</v>
+      </c>
+      <c r="S16" s="139">
+        <f t="shared" si="3"/>
+        <v>42.856000000000002</v>
+      </c>
+      <c r="T16" s="11"/>
+    </row>
+    <row r="17" spans="1:20" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="114"/>
+      <c r="B17" s="132"/>
       <c r="C17" s="78" t="s">
         <v>82</v>
       </c>
@@ -2938,33 +3148,44 @@
         <v>22</v>
       </c>
       <c r="K17" s="22">
-        <f>J17*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>1936.0000000000002</v>
       </c>
-      <c r="L17" s="40" t="s">
+      <c r="L17" s="8">
+        <f t="shared" si="0"/>
+        <v>2420</v>
+      </c>
+      <c r="M17" s="40" t="s">
         <v>225</v>
       </c>
-      <c r="M17" s="57">
+      <c r="N17" s="57">
         <v>0.249</v>
       </c>
-      <c r="N17" s="51">
-        <f t="shared" si="0"/>
+      <c r="O17" s="51">
+        <f t="shared" si="1"/>
         <v>5.4779999999999998</v>
       </c>
-      <c r="O17" s="57">
+      <c r="P17" s="57">
         <v>8.2890000000000005E-2</v>
       </c>
-      <c r="P17" s="51">
-        <f t="shared" si="1"/>
+      <c r="Q17" s="51">
+        <f t="shared" si="2"/>
         <v>160.47504000000004</v>
       </c>
-      <c r="Q17" s="23"/>
-    </row>
-    <row r="18" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R17" s="57">
+        <v>8.2890000000000005E-2</v>
+      </c>
+      <c r="S17" s="139">
+        <f t="shared" si="3"/>
+        <v>200.59380000000002</v>
+      </c>
+      <c r="T17" s="23"/>
+    </row>
+    <row r="18" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="113" t="s">
+      <c r="B18" s="131" t="s">
         <v>86</v>
       </c>
       <c r="C18" s="6" t="s">
@@ -2992,33 +3213,44 @@
         <v>1</v>
       </c>
       <c r="K18" s="8">
-        <f>J18*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L18" s="41" t="s">
+      <c r="L18" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M18" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="M18" s="55">
+      <c r="N18" s="55">
         <v>0.46</v>
       </c>
-      <c r="N18" s="52">
-        <f t="shared" si="0"/>
+      <c r="O18" s="52">
+        <f t="shared" si="1"/>
         <v>0.46</v>
       </c>
-      <c r="O18" s="55">
+      <c r="P18" s="55">
         <v>0.33839999999999998</v>
       </c>
-      <c r="P18" s="52">
-        <f t="shared" si="1"/>
+      <c r="Q18" s="52">
+        <f t="shared" si="2"/>
         <v>29.779199999999999</v>
       </c>
-      <c r="Q18" s="11"/>
-    </row>
-    <row r="19" spans="1:17" ht="102.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R18" s="55">
+        <v>0.33839999999999998</v>
+      </c>
+      <c r="S18" s="139">
+        <f t="shared" si="3"/>
+        <v>37.223999999999997</v>
+      </c>
+      <c r="T18" s="11"/>
+    </row>
+    <row r="19" spans="1:20" ht="102.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="111"/>
+      <c r="B19" s="133"/>
       <c r="C19" s="76" t="s">
         <v>91</v>
       </c>
@@ -3044,33 +3276,44 @@
         <v>45</v>
       </c>
       <c r="K19" s="16">
-        <f>J19*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>3960.0000000000005</v>
       </c>
-      <c r="L19" s="39" t="s">
+      <c r="L19" s="8">
+        <f t="shared" si="0"/>
+        <v>4950</v>
+      </c>
+      <c r="M19" s="39" t="s">
         <v>254</v>
       </c>
-      <c r="M19" s="56">
+      <c r="N19" s="56">
         <v>0.27100000000000002</v>
       </c>
-      <c r="N19" s="50">
-        <f t="shared" si="0"/>
+      <c r="O19" s="50">
+        <f t="shared" si="1"/>
         <v>12.195</v>
       </c>
-      <c r="O19" s="56">
+      <c r="P19" s="56">
         <v>0.11600000000000001</v>
       </c>
-      <c r="P19" s="50">
-        <f t="shared" si="1"/>
+      <c r="Q19" s="50">
+        <f t="shared" si="2"/>
         <v>459.36000000000007</v>
       </c>
-      <c r="Q19" s="24"/>
-    </row>
-    <row r="20" spans="1:17" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R19" s="56">
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="S19" s="139">
+        <f t="shared" si="3"/>
+        <v>574.20000000000005</v>
+      </c>
+      <c r="T19" s="24"/>
+    </row>
+    <row r="20" spans="1:20" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
-      <c r="B20" s="114"/>
+      <c r="B20" s="132"/>
       <c r="C20" s="19" t="s">
         <v>95</v>
       </c>
@@ -3096,33 +3339,44 @@
         <v>20</v>
       </c>
       <c r="K20" s="16">
-        <f>J20*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>1760.0000000000002</v>
       </c>
-      <c r="L20" s="40" t="s">
+      <c r="L20" s="8">
+        <f t="shared" si="0"/>
+        <v>2200</v>
+      </c>
+      <c r="M20" s="40" t="s">
         <v>225</v>
       </c>
-      <c r="M20" s="57">
+      <c r="N20" s="57">
         <v>0.36599999999999999</v>
       </c>
-      <c r="N20" s="51">
-        <f t="shared" si="0"/>
+      <c r="O20" s="51">
+        <f t="shared" si="1"/>
         <v>7.32</v>
       </c>
-      <c r="O20" s="57">
+      <c r="P20" s="57">
         <v>0.10525</v>
       </c>
-      <c r="P20" s="51">
-        <f t="shared" si="1"/>
+      <c r="Q20" s="51">
+        <f t="shared" si="2"/>
         <v>185.24</v>
       </c>
-      <c r="Q20" s="23"/>
-    </row>
-    <row r="21" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R20" s="57">
+        <v>0.10525</v>
+      </c>
+      <c r="S20" s="139">
+        <f t="shared" si="3"/>
+        <v>231.54999999999998</v>
+      </c>
+      <c r="T20" s="23"/>
+    </row>
+    <row r="21" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="113" t="s">
+      <c r="B21" s="131" t="s">
         <v>99</v>
       </c>
       <c r="C21" s="6" t="s">
@@ -3150,40 +3404,51 @@
         <v>1</v>
       </c>
       <c r="K21" s="8">
-        <f>J21*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L21" s="41" t="s">
+      <c r="L21" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M21" s="41" t="s">
         <v>247</v>
       </c>
-      <c r="M21" s="55">
+      <c r="N21" s="55">
         <v>0.18</v>
       </c>
-      <c r="N21" s="52">
-        <f t="shared" si="0"/>
+      <c r="O21" s="52">
+        <f t="shared" si="1"/>
         <v>0.18</v>
       </c>
-      <c r="O21" s="55">
+      <c r="P21" s="55">
         <v>0.10009999999999999</v>
       </c>
-      <c r="P21" s="52">
-        <f t="shared" si="1"/>
+      <c r="Q21" s="52">
+        <f t="shared" si="2"/>
         <v>8.8087999999999997</v>
       </c>
-      <c r="Q21" s="46"/>
-    </row>
-    <row r="22" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="55">
+        <v>0.10009999999999999</v>
+      </c>
+      <c r="S21" s="139">
+        <f t="shared" si="3"/>
+        <v>11.010999999999999</v>
+      </c>
+      <c r="T21" s="46"/>
+    </row>
+    <row r="22" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="111"/>
-      <c r="C22" s="122" t="s">
+      <c r="B22" s="133"/>
+      <c r="C22" s="110" t="s">
         <v>104</v>
       </c>
       <c r="D22" s="71" t="s">
         <v>105</v>
       </c>
-      <c r="E22" s="123" t="s">
+      <c r="E22" s="111" t="s">
         <v>239</v>
       </c>
       <c r="F22" s="71" t="s">
@@ -3198,37 +3463,48 @@
       <c r="I22" s="71" t="s">
         <v>240</v>
       </c>
-      <c r="J22" s="124">
+      <c r="J22" s="112">
         <v>1</v>
       </c>
-      <c r="K22" s="125">
-        <f>J22*80*1.1</f>
+      <c r="K22" s="113">
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L22" s="72" t="s">
+      <c r="L22" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M22" s="72" t="s">
         <v>237</v>
       </c>
-      <c r="M22" s="73">
+      <c r="N22" s="73">
         <v>0.2545</v>
       </c>
-      <c r="N22" s="73">
-        <f t="shared" si="0"/>
+      <c r="O22" s="73">
+        <f t="shared" si="1"/>
         <v>0.2545</v>
       </c>
-      <c r="O22" s="73">
+      <c r="P22" s="73">
         <v>0.18190000000000001</v>
       </c>
-      <c r="P22" s="73">
-        <f t="shared" si="1"/>
+      <c r="Q22" s="73">
+        <f t="shared" si="2"/>
         <v>16.007200000000001</v>
       </c>
-      <c r="Q22" s="126"/>
-    </row>
-    <row r="23" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R22" s="73">
+        <v>0.18190000000000001</v>
+      </c>
+      <c r="S22" s="139">
+        <f t="shared" si="3"/>
+        <v>20.009</v>
+      </c>
+      <c r="T22" s="114"/>
+    </row>
+    <row r="23" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="114"/>
+      <c r="B23" s="132"/>
       <c r="C23" s="19" t="s">
         <v>108</v>
       </c>
@@ -3254,29 +3530,40 @@
         <v>1</v>
       </c>
       <c r="K23" s="96">
-        <f>J23*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L23" s="40" t="s">
+      <c r="L23" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M23" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="M23" s="57">
+      <c r="N23" s="57">
         <v>1.92</v>
       </c>
-      <c r="N23" s="51">
-        <f t="shared" si="0"/>
+      <c r="O23" s="51">
+        <f t="shared" si="1"/>
         <v>1.92</v>
       </c>
-      <c r="O23" s="57">
+      <c r="P23" s="57">
         <v>1.44</v>
       </c>
-      <c r="P23" s="51">
-        <f t="shared" si="1"/>
+      <c r="Q23" s="51">
+        <f t="shared" si="2"/>
         <v>126.72</v>
       </c>
-      <c r="Q23" s="23"/>
-    </row>
-    <row r="24" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R23" s="57">
+        <v>1.44</v>
+      </c>
+      <c r="S23" s="139">
+        <f t="shared" si="3"/>
+        <v>158.4</v>
+      </c>
+      <c r="T23" s="23"/>
+    </row>
+    <row r="24" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -3308,33 +3595,44 @@
         <v>1</v>
       </c>
       <c r="K24" s="28">
-        <f>J24*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L24" s="47" t="s">
+      <c r="L24" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M24" s="47" t="s">
         <v>225</v>
       </c>
-      <c r="M24" s="59">
+      <c r="N24" s="59">
         <v>0.54</v>
       </c>
-      <c r="N24" s="53">
-        <f t="shared" si="0"/>
+      <c r="O24" s="53">
+        <f t="shared" si="1"/>
         <v>0.54</v>
       </c>
-      <c r="O24" s="59">
+      <c r="P24" s="59">
         <v>0.42399999999999999</v>
       </c>
-      <c r="P24" s="53">
-        <f t="shared" si="1"/>
+      <c r="Q24" s="53">
+        <f t="shared" si="2"/>
         <v>37.311999999999998</v>
       </c>
-      <c r="Q24" s="29"/>
-    </row>
-    <row r="25" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R24" s="59">
+        <v>0.42399999999999999</v>
+      </c>
+      <c r="S24" s="139">
+        <f t="shared" si="3"/>
+        <v>46.64</v>
+      </c>
+      <c r="T24" s="29"/>
+    </row>
+    <row r="25" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="110" t="s">
+      <c r="B25" s="127" t="s">
         <v>117</v>
       </c>
       <c r="C25" s="99" t="s">
@@ -3362,33 +3660,44 @@
         <v>1</v>
       </c>
       <c r="K25" s="102">
-        <f>J25*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L25" s="103" t="s">
+      <c r="L25" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M25" s="103" t="s">
         <v>247</v>
       </c>
-      <c r="M25" s="104">
+      <c r="N25" s="104">
         <v>0.9</v>
       </c>
-      <c r="N25" s="105">
-        <f t="shared" si="0"/>
+      <c r="O25" s="105">
+        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
-      <c r="O25" s="104">
+      <c r="P25" s="104">
         <v>0.7823</v>
       </c>
-      <c r="P25" s="105">
-        <f t="shared" si="1"/>
+      <c r="Q25" s="105">
+        <f t="shared" si="2"/>
         <v>68.842399999999998</v>
       </c>
-      <c r="Q25" s="106"/>
-    </row>
-    <row r="26" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R25" s="104">
+        <v>0.7823</v>
+      </c>
+      <c r="S25" s="139">
+        <f t="shared" si="3"/>
+        <v>86.052999999999997</v>
+      </c>
+      <c r="T25" s="106"/>
+    </row>
+    <row r="26" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="112"/>
+      <c r="B26" s="128"/>
       <c r="C26" s="80" t="s">
         <v>122</v>
       </c>
@@ -3414,54 +3723,65 @@
         <v>1</v>
       </c>
       <c r="K26" s="84">
-        <f>J26*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L26" s="85" t="s">
+      <c r="L26" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M26" s="85" t="s">
         <v>225</v>
       </c>
-      <c r="M26" s="86">
+      <c r="N26" s="86">
         <v>0.48</v>
       </c>
-      <c r="N26" s="87">
-        <f t="shared" si="0"/>
+      <c r="O26" s="87">
+        <f t="shared" si="1"/>
         <v>0.48</v>
       </c>
-      <c r="O26" s="86">
+      <c r="P26" s="86">
         <v>0.43840000000000001</v>
       </c>
-      <c r="P26" s="87">
-        <f t="shared" si="1"/>
+      <c r="Q26" s="87">
+        <f t="shared" si="2"/>
         <v>38.5792</v>
       </c>
-      <c r="Q26" s="88"/>
-    </row>
-    <row r="27" spans="1:17" ht="115.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R26" s="86">
+        <v>0.43840000000000001</v>
+      </c>
+      <c r="S26" s="139">
+        <f t="shared" si="3"/>
+        <v>48.224000000000004</v>
+      </c>
+      <c r="T26" s="88"/>
+    </row>
+    <row r="27" spans="1:20" ht="115.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="117" t="s">
+      <c r="B27" s="134" t="s">
         <v>126</v>
       </c>
-      <c r="C27" s="128" t="s">
+      <c r="C27" s="116" t="s">
         <v>127</v>
       </c>
-      <c r="D27" s="129" t="s">
+      <c r="D27" s="117" t="s">
         <v>255</v>
       </c>
-      <c r="E27" s="130" t="s">
+      <c r="E27" s="118" t="s">
         <v>128</v>
       </c>
-      <c r="F27" s="130" t="s">
+      <c r="F27" s="118" t="s">
         <v>129</v>
       </c>
-      <c r="G27" s="130" t="s">
+      <c r="G27" s="118" t="s">
         <v>24</v>
       </c>
-      <c r="H27" s="130" t="s">
+      <c r="H27" s="118" t="s">
         <v>240</v>
       </c>
-      <c r="I27" s="130" t="s">
+      <c r="I27" s="118" t="s">
         <v>130</v>
       </c>
       <c r="J27" s="9">
@@ -3469,33 +3789,44 @@
         <v>52</v>
       </c>
       <c r="K27" s="8">
-        <f>J27*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>4576</v>
       </c>
-      <c r="L27" s="41" t="s">
+      <c r="L27" s="8">
+        <f t="shared" si="0"/>
+        <v>5720</v>
+      </c>
+      <c r="M27" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="M27" s="55">
+      <c r="N27" s="55">
         <v>1.6E-2</v>
       </c>
-      <c r="N27" s="127">
-        <f>M27*J27</f>
+      <c r="O27" s="115">
+        <f>N27*J27</f>
         <v>0.83200000000000007</v>
       </c>
-      <c r="O27" s="55">
+      <c r="P27" s="55">
         <v>2.5899999999999999E-3</v>
       </c>
-      <c r="P27" s="52">
-        <f t="shared" si="1"/>
+      <c r="Q27" s="52">
+        <f t="shared" si="2"/>
         <v>11.851839999999999</v>
       </c>
-      <c r="Q27" s="11"/>
-    </row>
-    <row r="28" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R27" s="55">
+        <v>2.5899999999999999E-3</v>
+      </c>
+      <c r="S27" s="139">
+        <f t="shared" si="3"/>
+        <v>14.8148</v>
+      </c>
+      <c r="T27" s="11"/>
+    </row>
+    <row r="28" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>26</v>
       </c>
-      <c r="B28" s="118"/>
+      <c r="B28" s="135"/>
       <c r="C28" s="12" t="s">
         <v>131</v>
       </c>
@@ -3521,33 +3852,44 @@
         <v>1</v>
       </c>
       <c r="K28" s="16">
-        <f>J28*80*1.1</f>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
-      <c r="L28" s="39" t="s">
+      <c r="L28" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M28" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="M28" s="56">
+      <c r="N28" s="56">
         <v>0.1</v>
       </c>
-      <c r="N28" s="50">
-        <f t="shared" si="0"/>
+      <c r="O28" s="50">
+        <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O28" s="56">
+      <c r="P28" s="56">
         <v>1.6E-2</v>
       </c>
-      <c r="P28" s="50">
-        <f t="shared" si="1"/>
+      <c r="Q28" s="50">
+        <f t="shared" si="2"/>
         <v>1.4079999999999999</v>
       </c>
-      <c r="Q28" s="17"/>
-    </row>
-    <row r="29" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R28" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="S28" s="139">
+        <f t="shared" si="3"/>
+        <v>1.76</v>
+      </c>
+      <c r="T28" s="17"/>
+    </row>
+    <row r="29" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>27</v>
       </c>
-      <c r="B29" s="118"/>
+      <c r="B29" s="135"/>
       <c r="C29" s="12" t="s">
         <v>137</v>
       </c>
@@ -3573,33 +3915,44 @@
         <v>5</v>
       </c>
       <c r="K29" s="16">
-        <f t="shared" ref="K29:K40" si="3">J29*80*1.1</f>
+        <f t="shared" ref="K29:K40" si="6">J29*80*1.1</f>
         <v>440.00000000000006</v>
       </c>
-      <c r="L29" s="39" t="s">
+      <c r="L29" s="8">
+        <f t="shared" si="0"/>
+        <v>550</v>
+      </c>
+      <c r="M29" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="M29" s="56">
+      <c r="N29" s="56">
         <v>0.1</v>
       </c>
-      <c r="N29" s="50">
-        <f t="shared" si="0"/>
+      <c r="O29" s="50">
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="O29" s="56">
+      <c r="P29" s="56">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="P29" s="50">
-        <f t="shared" si="1"/>
+      <c r="Q29" s="50">
+        <f t="shared" si="2"/>
         <v>3.5200000000000005</v>
       </c>
-      <c r="Q29" s="17"/>
-    </row>
-    <row r="30" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R29" s="56">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="S29" s="139">
+        <f t="shared" si="3"/>
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="T29" s="17"/>
+    </row>
+    <row r="30" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" s="118"/>
+      <c r="B30" s="135"/>
       <c r="C30" s="12" t="s">
         <v>142</v>
       </c>
@@ -3625,33 +3978,44 @@
         <v>1</v>
       </c>
       <c r="K30" s="16">
+        <f t="shared" si="6"/>
+        <v>88</v>
+      </c>
+      <c r="L30" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M30" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N30" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O30" s="50">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="P30" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="Q30" s="50">
+        <f t="shared" si="2"/>
+        <v>1.4079999999999999</v>
+      </c>
+      <c r="R30" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="S30" s="139">
         <f t="shared" si="3"/>
-        <v>88</v>
-      </c>
-      <c r="L30" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M30" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N30" s="50">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-      <c r="O30" s="56">
-        <v>1.6E-2</v>
-      </c>
-      <c r="P30" s="50">
-        <f t="shared" si="1"/>
-        <v>1.4079999999999999</v>
-      </c>
-      <c r="Q30" s="17"/>
-    </row>
-    <row r="31" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.76</v>
+      </c>
+      <c r="T30" s="17"/>
+    </row>
+    <row r="31" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="118"/>
+      <c r="B31" s="135"/>
       <c r="C31" s="12" t="s">
         <v>146</v>
       </c>
@@ -3677,33 +4041,44 @@
         <v>2</v>
       </c>
       <c r="K31" s="16">
+        <f t="shared" si="6"/>
+        <v>176</v>
+      </c>
+      <c r="L31" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M31" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N31" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O31" s="50">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="P31" s="56">
+        <v>6.6E-3</v>
+      </c>
+      <c r="Q31" s="50">
+        <f t="shared" si="2"/>
+        <v>1.1616</v>
+      </c>
+      <c r="R31" s="56">
+        <v>6.6E-3</v>
+      </c>
+      <c r="S31" s="139">
         <f t="shared" si="3"/>
-        <v>176</v>
-      </c>
-      <c r="L31" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M31" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N31" s="50">
-        <f t="shared" si="0"/>
-        <v>0.2</v>
-      </c>
-      <c r="O31" s="56">
-        <v>6.6E-3</v>
-      </c>
-      <c r="P31" s="50">
-        <f t="shared" si="1"/>
-        <v>1.1616</v>
-      </c>
-      <c r="Q31" s="17"/>
-    </row>
-    <row r="32" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.452</v>
+      </c>
+      <c r="T31" s="17"/>
+    </row>
+    <row r="32" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="118"/>
+      <c r="B32" s="135"/>
       <c r="C32" s="12" t="s">
         <v>150</v>
       </c>
@@ -3729,33 +4104,44 @@
         <v>1</v>
       </c>
       <c r="K32" s="16">
+        <f t="shared" si="6"/>
+        <v>88</v>
+      </c>
+      <c r="L32" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M32" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N32" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O32" s="50">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="P32" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="Q32" s="50">
+        <f t="shared" si="2"/>
+        <v>1.4079999999999999</v>
+      </c>
+      <c r="R32" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="S32" s="139">
         <f t="shared" si="3"/>
-        <v>88</v>
-      </c>
-      <c r="L32" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M32" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N32" s="50">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-      <c r="O32" s="56">
-        <v>1.6E-2</v>
-      </c>
-      <c r="P32" s="50">
-        <f t="shared" si="1"/>
-        <v>1.4079999999999999</v>
-      </c>
-      <c r="Q32" s="17"/>
-    </row>
-    <row r="33" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.76</v>
+      </c>
+      <c r="T32" s="17"/>
+    </row>
+    <row r="33" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="118"/>
+      <c r="B33" s="135"/>
       <c r="C33" s="12" t="s">
         <v>154</v>
       </c>
@@ -3781,33 +4167,44 @@
         <v>1</v>
       </c>
       <c r="K33" s="16">
+        <f t="shared" si="6"/>
+        <v>88</v>
+      </c>
+      <c r="L33" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M33" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N33" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O33" s="50">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="P33" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="Q33" s="50">
+        <f t="shared" si="2"/>
+        <v>1.4079999999999999</v>
+      </c>
+      <c r="R33" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="S33" s="139">
         <f t="shared" si="3"/>
-        <v>88</v>
-      </c>
-      <c r="L33" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M33" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N33" s="50">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-      <c r="O33" s="56">
-        <v>1.6E-2</v>
-      </c>
-      <c r="P33" s="50">
-        <f t="shared" si="1"/>
-        <v>1.4079999999999999</v>
-      </c>
-      <c r="Q33" s="17"/>
-    </row>
-    <row r="34" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.76</v>
+      </c>
+      <c r="T33" s="17"/>
+    </row>
+    <row r="34" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>32</v>
       </c>
-      <c r="B34" s="118"/>
+      <c r="B34" s="135"/>
       <c r="C34" s="12" t="s">
         <v>158</v>
       </c>
@@ -3833,33 +4230,44 @@
         <v>5</v>
       </c>
       <c r="K34" s="16">
+        <f t="shared" si="6"/>
+        <v>440.00000000000006</v>
+      </c>
+      <c r="L34" s="8">
+        <f t="shared" si="0"/>
+        <v>550</v>
+      </c>
+      <c r="M34" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N34" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O34" s="50">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="P34" s="56">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="Q34" s="50">
+        <f t="shared" si="2"/>
+        <v>3.9600000000000004</v>
+      </c>
+      <c r="R34" s="56">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="S34" s="139">
         <f t="shared" si="3"/>
-        <v>440.00000000000006</v>
-      </c>
-      <c r="L34" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M34" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N34" s="50">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-      <c r="O34" s="56">
-        <v>8.9999999999999993E-3</v>
-      </c>
-      <c r="P34" s="50">
-        <f t="shared" si="1"/>
-        <v>3.9600000000000004</v>
-      </c>
-      <c r="Q34" s="17"/>
-    </row>
-    <row r="35" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4.9499999999999993</v>
+      </c>
+      <c r="T34" s="17"/>
+    </row>
+    <row r="35" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="118"/>
+      <c r="B35" s="135"/>
       <c r="C35" s="12" t="s">
         <v>163</v>
       </c>
@@ -3885,33 +4293,44 @@
         <v>2</v>
       </c>
       <c r="K35" s="16">
+        <f t="shared" si="6"/>
+        <v>176</v>
+      </c>
+      <c r="L35" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M35" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N35" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O35" s="50">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="P35" s="56">
+        <v>6.6E-3</v>
+      </c>
+      <c r="Q35" s="50">
+        <f t="shared" si="2"/>
+        <v>1.1616</v>
+      </c>
+      <c r="R35" s="56">
+        <v>6.6E-3</v>
+      </c>
+      <c r="S35" s="139">
         <f t="shared" si="3"/>
-        <v>176</v>
-      </c>
-      <c r="L35" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M35" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N35" s="50">
-        <f t="shared" si="0"/>
-        <v>0.2</v>
-      </c>
-      <c r="O35" s="56">
-        <v>6.6E-3</v>
-      </c>
-      <c r="P35" s="50">
-        <f t="shared" si="1"/>
-        <v>1.1616</v>
-      </c>
-      <c r="Q35" s="48"/>
-    </row>
-    <row r="36" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.452</v>
+      </c>
+      <c r="T35" s="48"/>
+    </row>
+    <row r="36" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>35</v>
       </c>
-      <c r="B36" s="118"/>
+      <c r="B36" s="135"/>
       <c r="C36" s="12" t="s">
         <v>167</v>
       </c>
@@ -3937,33 +4356,44 @@
         <v>4</v>
       </c>
       <c r="K36" s="16">
+        <f t="shared" si="6"/>
+        <v>352</v>
+      </c>
+      <c r="L36" s="8">
+        <f t="shared" si="0"/>
+        <v>440</v>
+      </c>
+      <c r="M36" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N36" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O36" s="50">
+        <f t="shared" si="1"/>
+        <v>0.4</v>
+      </c>
+      <c r="P36" s="56">
+        <v>6.6E-3</v>
+      </c>
+      <c r="Q36" s="50">
+        <f t="shared" si="2"/>
+        <v>2.3231999999999999</v>
+      </c>
+      <c r="R36" s="56">
+        <v>6.6E-3</v>
+      </c>
+      <c r="S36" s="139">
         <f t="shared" si="3"/>
-        <v>352</v>
-      </c>
-      <c r="L36" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M36" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N36" s="50">
-        <f t="shared" si="0"/>
-        <v>0.4</v>
-      </c>
-      <c r="O36" s="56">
-        <v>6.6E-3</v>
-      </c>
-      <c r="P36" s="50">
-        <f t="shared" si="1"/>
-        <v>2.3231999999999999</v>
-      </c>
-      <c r="Q36" s="17"/>
-    </row>
-    <row r="37" spans="1:17" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2.9039999999999999</v>
+      </c>
+      <c r="T36" s="17"/>
+    </row>
+    <row r="37" spans="1:20" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>36</v>
       </c>
-      <c r="B37" s="118"/>
+      <c r="B37" s="135"/>
       <c r="C37" s="76" t="s">
         <v>171</v>
       </c>
@@ -3989,33 +4419,44 @@
         <v>20</v>
       </c>
       <c r="K37" s="16">
+        <f t="shared" si="6"/>
+        <v>1760.0000000000002</v>
+      </c>
+      <c r="L37" s="8">
+        <f t="shared" si="0"/>
+        <v>2200</v>
+      </c>
+      <c r="M37" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N37" s="56">
+        <v>1.6E-2</v>
+      </c>
+      <c r="O37" s="50">
+        <f t="shared" si="1"/>
+        <v>0.32</v>
+      </c>
+      <c r="P37" s="56">
+        <v>2.99E-3</v>
+      </c>
+      <c r="Q37" s="50">
+        <f t="shared" si="2"/>
+        <v>5.2624000000000004</v>
+      </c>
+      <c r="R37" s="56">
+        <v>2.99E-3</v>
+      </c>
+      <c r="S37" s="139">
         <f t="shared" si="3"/>
-        <v>1760.0000000000002</v>
-      </c>
-      <c r="L37" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M37" s="56">
-        <v>1.6E-2</v>
-      </c>
-      <c r="N37" s="50">
-        <f t="shared" si="0"/>
-        <v>0.32</v>
-      </c>
-      <c r="O37" s="56">
-        <v>2.99E-3</v>
-      </c>
-      <c r="P37" s="50">
-        <f t="shared" si="1"/>
-        <v>5.2624000000000004</v>
-      </c>
-      <c r="Q37" s="17"/>
-    </row>
-    <row r="38" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>6.5780000000000003</v>
+      </c>
+      <c r="T37" s="17"/>
+    </row>
+    <row r="38" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>37</v>
       </c>
-      <c r="B38" s="118"/>
+      <c r="B38" s="135"/>
       <c r="C38" s="12" t="s">
         <v>175</v>
       </c>
@@ -4041,33 +4482,44 @@
         <v>1</v>
       </c>
       <c r="K38" s="16">
+        <f t="shared" si="6"/>
+        <v>88</v>
+      </c>
+      <c r="L38" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M38" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N38" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O38" s="50">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="P38" s="56">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="Q38" s="50">
+        <f t="shared" si="2"/>
+        <v>1.3199999999999998</v>
+      </c>
+      <c r="R38" s="56">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="S38" s="139">
         <f t="shared" si="3"/>
-        <v>88</v>
-      </c>
-      <c r="L38" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M38" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N38" s="50">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-      <c r="O38" s="56">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="P38" s="50">
-        <f t="shared" si="1"/>
-        <v>1.3199999999999998</v>
-      </c>
-      <c r="Q38" s="17"/>
-    </row>
-    <row r="39" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.65</v>
+      </c>
+      <c r="T38" s="17"/>
+    </row>
+    <row r="39" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>38</v>
       </c>
-      <c r="B39" s="118"/>
+      <c r="B39" s="135"/>
       <c r="C39" s="12" t="s">
         <v>179</v>
       </c>
@@ -4093,33 +4545,44 @@
         <v>4</v>
       </c>
       <c r="K39" s="16">
+        <f t="shared" si="6"/>
+        <v>352</v>
+      </c>
+      <c r="L39" s="8">
+        <f t="shared" si="0"/>
+        <v>440</v>
+      </c>
+      <c r="M39" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="N39" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="O39" s="50">
+        <f t="shared" si="1"/>
+        <v>0.4</v>
+      </c>
+      <c r="P39" s="56">
+        <v>5.4000000000000003E-3</v>
+      </c>
+      <c r="Q39" s="50">
+        <f t="shared" si="2"/>
+        <v>1.9008</v>
+      </c>
+      <c r="R39" s="56">
+        <v>5.4000000000000003E-3</v>
+      </c>
+      <c r="S39" s="139">
         <f t="shared" si="3"/>
-        <v>352</v>
-      </c>
-      <c r="L39" s="39" t="s">
-        <v>225</v>
-      </c>
-      <c r="M39" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="N39" s="50">
-        <f t="shared" si="0"/>
-        <v>0.4</v>
-      </c>
-      <c r="O39" s="56">
-        <v>5.4000000000000003E-3</v>
-      </c>
-      <c r="P39" s="50">
-        <f t="shared" si="1"/>
-        <v>1.9008</v>
-      </c>
-      <c r="Q39" s="17"/>
-    </row>
-    <row r="40" spans="1:17" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2.3760000000000003</v>
+      </c>
+      <c r="T39" s="17"/>
+    </row>
+    <row r="40" spans="1:20" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>39</v>
       </c>
-      <c r="B40" s="119"/>
+      <c r="B40" s="136"/>
       <c r="C40" s="68" t="s">
         <v>135</v>
       </c>
@@ -4145,52 +4608,63 @@
         <v>22</v>
       </c>
       <c r="K40" s="16">
+        <f t="shared" si="6"/>
+        <v>1936.0000000000002</v>
+      </c>
+      <c r="L40" s="8">
+        <f t="shared" si="0"/>
+        <v>2420</v>
+      </c>
+      <c r="M40" s="90" t="s">
+        <v>225</v>
+      </c>
+      <c r="N40" s="91">
+        <v>0.11799999999999999</v>
+      </c>
+      <c r="O40" s="92">
+        <f t="shared" si="1"/>
+        <v>2.5960000000000001</v>
+      </c>
+      <c r="P40" s="91">
+        <v>1.9349999999999999E-2</v>
+      </c>
+      <c r="Q40" s="92">
+        <f t="shared" si="2"/>
+        <v>37.461600000000004</v>
+      </c>
+      <c r="R40" s="91">
+        <v>1.9349999999999999E-2</v>
+      </c>
+      <c r="S40" s="139">
         <f t="shared" si="3"/>
-        <v>1936.0000000000002</v>
-      </c>
-      <c r="L40" s="90" t="s">
-        <v>225</v>
-      </c>
-      <c r="M40" s="91">
-        <v>0.11799999999999999</v>
-      </c>
-      <c r="N40" s="92">
-        <f t="shared" si="0"/>
-        <v>2.5960000000000001</v>
-      </c>
-      <c r="O40" s="91">
-        <v>1.9349999999999999E-2</v>
-      </c>
-      <c r="P40" s="92">
-        <f t="shared" si="1"/>
-        <v>37.461600000000004</v>
-      </c>
-      <c r="Q40" s="93"/>
-    </row>
-    <row r="41" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>46.826999999999998</v>
+      </c>
+      <c r="T40" s="93"/>
+    </row>
+    <row r="41" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>40</v>
       </c>
       <c r="B41" s="107" t="s">
         <v>184</v>
       </c>
-      <c r="C41" s="135" t="s">
+      <c r="C41" s="123" t="s">
         <v>185</v>
       </c>
-      <c r="D41" s="136" t="s">
+      <c r="D41" s="124" t="s">
         <v>186</v>
       </c>
-      <c r="E41" s="136" t="s">
+      <c r="E41" s="124" t="s">
         <v>239</v>
       </c>
-      <c r="F41" s="136" t="s">
+      <c r="F41" s="124" t="s">
         <v>187</v>
       </c>
-      <c r="G41" s="136" t="s">
+      <c r="G41" s="124" t="s">
         <v>188</v>
       </c>
-      <c r="H41" s="137"/>
-      <c r="I41" s="138" t="s">
+      <c r="H41" s="125"/>
+      <c r="I41" s="126" t="s">
         <v>240</v>
       </c>
       <c r="J41" s="95">
@@ -4200,30 +4674,41 @@
         <f>J41*80*1.1</f>
         <v>88</v>
       </c>
-      <c r="L41" s="131" t="s">
+      <c r="L41" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M41" s="119" t="s">
         <v>237</v>
       </c>
-      <c r="M41" s="132">
+      <c r="N41" s="120">
         <v>0.13389999999999999</v>
       </c>
-      <c r="N41" s="133">
-        <f t="shared" si="0"/>
+      <c r="O41" s="121">
+        <f t="shared" si="1"/>
         <v>0.13389999999999999</v>
       </c>
-      <c r="O41" s="132">
+      <c r="P41" s="120">
         <v>0.1072</v>
       </c>
-      <c r="P41" s="133">
-        <f t="shared" si="1"/>
+      <c r="Q41" s="121">
+        <f t="shared" si="2"/>
         <v>9.4336000000000002</v>
       </c>
-      <c r="Q41" s="134"/>
-    </row>
-    <row r="42" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R41" s="120">
+        <v>0.1072</v>
+      </c>
+      <c r="S41" s="139">
+        <f t="shared" si="3"/>
+        <v>11.792</v>
+      </c>
+      <c r="T41" s="122"/>
+    </row>
+    <row r="42" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>41</v>
       </c>
-      <c r="B42" s="110" t="s">
+      <c r="B42" s="127" t="s">
         <v>189</v>
       </c>
       <c r="C42" s="99" t="s">
@@ -4254,30 +4739,41 @@
         <f>J42*80*1.1</f>
         <v>176</v>
       </c>
-      <c r="L42" s="103" t="s">
+      <c r="L42" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M42" s="103" t="s">
         <v>236</v>
       </c>
-      <c r="M42" s="104">
+      <c r="N42" s="104">
         <v>0.66876000000000002</v>
       </c>
-      <c r="N42" s="105">
-        <f t="shared" si="0"/>
+      <c r="O42" s="105">
+        <f t="shared" si="1"/>
         <v>1.33752</v>
       </c>
-      <c r="O42" s="104">
+      <c r="P42" s="104">
         <v>0.42204000000000003</v>
       </c>
-      <c r="P42" s="105">
-        <f t="shared" si="1"/>
+      <c r="Q42" s="105">
+        <f t="shared" si="2"/>
         <v>74.279040000000009</v>
       </c>
-      <c r="Q42" s="106"/>
-    </row>
-    <row r="43" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R42" s="104">
+        <v>0.42204000000000003</v>
+      </c>
+      <c r="S42" s="139">
+        <f t="shared" si="3"/>
+        <v>92.848800000000011</v>
+      </c>
+      <c r="T42" s="106"/>
+    </row>
+    <row r="43" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>42</v>
       </c>
-      <c r="B43" s="111"/>
+      <c r="B43" s="133"/>
       <c r="C43" s="12" t="s">
         <v>194</v>
       </c>
@@ -4306,30 +4802,41 @@
         <f>J43*80*1.1</f>
         <v>88</v>
       </c>
-      <c r="L43" s="39" t="s">
+      <c r="L43" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M43" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="M43" s="56">
+      <c r="N43" s="56">
         <v>0.65</v>
       </c>
-      <c r="N43" s="50">
-        <f t="shared" si="0"/>
+      <c r="O43" s="50">
+        <f t="shared" si="1"/>
         <v>0.65</v>
       </c>
-      <c r="O43" s="56">
+      <c r="P43" s="56">
         <v>0.57199999999999995</v>
       </c>
-      <c r="P43" s="50">
-        <f t="shared" si="1"/>
+      <c r="Q43" s="50">
+        <f t="shared" si="2"/>
         <v>50.335999999999999</v>
       </c>
-      <c r="Q43" s="17"/>
-    </row>
-    <row r="44" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R43" s="56">
+        <v>0.57199999999999995</v>
+      </c>
+      <c r="S43" s="139">
+        <f t="shared" si="3"/>
+        <v>62.919999999999995</v>
+      </c>
+      <c r="T43" s="17"/>
+    </row>
+    <row r="44" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>43</v>
       </c>
-      <c r="B44" s="111"/>
+      <c r="B44" s="133"/>
       <c r="C44" s="12" t="s">
         <v>198</v>
       </c>
@@ -4355,33 +4862,44 @@
         <v>1</v>
       </c>
       <c r="K44" s="16">
-        <f t="shared" ref="K44:K45" si="4">J44*80*1.1</f>
+        <f t="shared" ref="K44:K45" si="7">J44*80*1.1</f>
         <v>88</v>
       </c>
-      <c r="L44" s="39" t="s">
+      <c r="L44" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M44" s="39" t="s">
         <v>236</v>
       </c>
-      <c r="M44" s="58">
+      <c r="N44" s="58">
         <v>22.08108</v>
       </c>
-      <c r="N44" s="50">
-        <f t="shared" si="0"/>
+      <c r="O44" s="50">
+        <f t="shared" si="1"/>
         <v>22.08108</v>
       </c>
-      <c r="O44" s="58">
+      <c r="P44" s="58">
         <v>18.247319999999998</v>
       </c>
-      <c r="P44" s="50">
-        <f t="shared" si="1"/>
+      <c r="Q44" s="50">
+        <f t="shared" si="2"/>
         <v>1605.7641599999999</v>
       </c>
-      <c r="Q44" s="17"/>
-    </row>
-    <row r="45" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R44" s="58">
+        <v>18.247319999999998</v>
+      </c>
+      <c r="S44" s="139">
+        <f t="shared" si="3"/>
+        <v>2007.2051999999999</v>
+      </c>
+      <c r="T44" s="17"/>
+    </row>
+    <row r="45" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>44</v>
       </c>
-      <c r="B45" s="112"/>
+      <c r="B45" s="128"/>
       <c r="C45" s="80" t="s">
         <v>201</v>
       </c>
@@ -4407,33 +4925,44 @@
         <v>5</v>
       </c>
       <c r="K45" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>440.00000000000006</v>
       </c>
-      <c r="L45" s="85" t="s">
+      <c r="L45" s="8">
+        <f t="shared" si="0"/>
+        <v>550</v>
+      </c>
+      <c r="M45" s="85" t="s">
         <v>251</v>
       </c>
-      <c r="M45" s="98">
+      <c r="N45" s="98">
         <v>1.22</v>
       </c>
-      <c r="N45" s="87">
-        <f t="shared" si="0"/>
+      <c r="O45" s="87">
+        <f t="shared" si="1"/>
         <v>6.1</v>
       </c>
-      <c r="O45" s="98">
+      <c r="P45" s="98">
         <v>0.51</v>
       </c>
-      <c r="P45" s="87">
-        <f t="shared" si="1"/>
+      <c r="Q45" s="87">
+        <f t="shared" si="2"/>
         <v>224.40000000000003</v>
       </c>
-      <c r="Q45" s="88"/>
-    </row>
-    <row r="46" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R45" s="98">
+        <v>0.51</v>
+      </c>
+      <c r="S45" s="139">
+        <f t="shared" si="3"/>
+        <v>280.5</v>
+      </c>
+      <c r="T45" s="88"/>
+    </row>
+    <row r="46" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>45</v>
       </c>
-      <c r="B46" s="113" t="s">
+      <c r="B46" s="131" t="s">
         <v>205</v>
       </c>
       <c r="C46" s="6" t="s">
@@ -4464,30 +4993,41 @@
         <f>J46*80*1.1</f>
         <v>88</v>
       </c>
-      <c r="L46" s="41" t="s">
+      <c r="L46" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M46" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="M46" s="55">
+      <c r="N46" s="55">
         <v>0.44</v>
       </c>
-      <c r="N46" s="52">
-        <f t="shared" si="0"/>
+      <c r="O46" s="52">
+        <f t="shared" si="1"/>
         <v>0.44</v>
       </c>
-      <c r="O46" s="55">
+      <c r="P46" s="55">
         <v>0.32819999999999999</v>
       </c>
-      <c r="P46" s="52">
-        <f t="shared" si="1"/>
+      <c r="Q46" s="52">
+        <f t="shared" si="2"/>
         <v>28.881599999999999</v>
       </c>
-      <c r="Q46" s="11"/>
-    </row>
-    <row r="47" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R46" s="55">
+        <v>0.32819999999999999</v>
+      </c>
+      <c r="S46" s="139">
+        <f t="shared" si="3"/>
+        <v>36.101999999999997</v>
+      </c>
+      <c r="T46" s="11"/>
+    </row>
+    <row r="47" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>46</v>
       </c>
-      <c r="B47" s="111"/>
+      <c r="B47" s="133"/>
       <c r="C47" s="43" t="s">
         <v>210</v>
       </c>
@@ -4516,30 +5056,41 @@
         <f>J47*80*1.1</f>
         <v>88</v>
       </c>
-      <c r="L47" s="42" t="s">
+      <c r="L47" s="8">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+      <c r="M47" s="42" t="s">
         <v>225</v>
       </c>
-      <c r="M47" s="60">
+      <c r="N47" s="60">
         <v>6.06</v>
       </c>
-      <c r="N47" s="54">
-        <f t="shared" si="0"/>
+      <c r="O47" s="54">
+        <f t="shared" si="1"/>
         <v>6.06</v>
       </c>
-      <c r="O47" s="60">
+      <c r="P47" s="60">
         <v>5.51</v>
       </c>
-      <c r="P47" s="54">
-        <f t="shared" si="1"/>
+      <c r="Q47" s="54">
+        <f t="shared" si="2"/>
         <v>484.88</v>
       </c>
-      <c r="Q47" s="49"/>
-    </row>
-    <row r="48" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R47" s="60">
+        <v>5.51</v>
+      </c>
+      <c r="S47" s="139">
+        <f t="shared" si="3"/>
+        <v>606.1</v>
+      </c>
+      <c r="T47" s="49"/>
+    </row>
+    <row r="48" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>47</v>
       </c>
-      <c r="B48" s="111"/>
+      <c r="B48" s="133"/>
       <c r="C48" s="12" t="s">
         <v>214</v>
       </c>
@@ -4565,33 +5116,44 @@
         <v>2</v>
       </c>
       <c r="K48" s="31">
-        <f t="shared" ref="K48:K49" si="5">J48*80*1.1</f>
+        <f t="shared" ref="K48:K49" si="8">J48*80*1.1</f>
         <v>176</v>
       </c>
-      <c r="L48" s="39" t="s">
+      <c r="L48" s="8">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="M48" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="M48" s="56">
+      <c r="N48" s="56">
         <v>0.75</v>
       </c>
-      <c r="N48" s="50">
-        <f t="shared" si="0"/>
+      <c r="O48" s="50">
+        <f t="shared" si="1"/>
         <v>1.5</v>
       </c>
-      <c r="O48" s="56">
+      <c r="P48" s="56">
         <v>0.51670000000000005</v>
       </c>
-      <c r="P48" s="50">
-        <f t="shared" si="1"/>
+      <c r="Q48" s="50">
+        <f t="shared" si="2"/>
         <v>90.939200000000014</v>
       </c>
-      <c r="Q48" s="17"/>
-    </row>
-    <row r="49" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R48" s="56">
+        <v>0.51670000000000005</v>
+      </c>
+      <c r="S48" s="139">
+        <f t="shared" si="3"/>
+        <v>113.67400000000001</v>
+      </c>
+      <c r="T48" s="17"/>
+    </row>
+    <row r="49" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>48</v>
       </c>
-      <c r="B49" s="114"/>
+      <c r="B49" s="132"/>
       <c r="C49" s="45" t="s">
         <v>218</v>
       </c>
@@ -4617,84 +5179,102 @@
         <v>7</v>
       </c>
       <c r="K49" s="31">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>616</v>
       </c>
-      <c r="L49" s="33"/>
+      <c r="L49" s="8">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
       <c r="M49" s="33"/>
       <c r="N49" s="33"/>
       <c r="O49" s="33"/>
       <c r="P49" s="33"/>
-      <c r="Q49" s="35"/>
-    </row>
-    <row r="50" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q49" s="33"/>
+      <c r="R49" s="140"/>
+      <c r="S49" s="140"/>
+      <c r="T49" s="35"/>
+    </row>
+    <row r="50" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B50" s="36"/>
-      <c r="J50" s="115" t="s">
+      <c r="J50" s="137" t="s">
         <v>221</v>
       </c>
-      <c r="K50" s="115"/>
-      <c r="L50" s="115"/>
-      <c r="M50" s="115"/>
-      <c r="N50" s="61"/>
+      <c r="K50" s="137"/>
+      <c r="L50" s="137"/>
+      <c r="M50" s="137"/>
+      <c r="N50" s="137"/>
       <c r="O50" s="61"/>
-      <c r="P50" s="62">
-        <f>SUM(P3:P48)</f>
+      <c r="P50" s="61"/>
+      <c r="Q50" s="62">
+        <f>SUM(Q3:Q48)</f>
         <v>4334.784959999999</v>
       </c>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R50" s="62"/>
+      <c r="S50" s="62">
+        <f>SUM(S3:S49)</f>
+        <v>5418.481200000002</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B51" s="36"/>
-      <c r="J51" s="116" t="s">
+      <c r="J51" s="138" t="s">
         <v>222</v>
       </c>
-      <c r="K51" s="116"/>
-      <c r="L51" s="116"/>
-      <c r="M51" s="116"/>
-      <c r="N51" s="37">
-        <f>SUM(N3:N48)</f>
+      <c r="K51" s="138"/>
+      <c r="L51" s="138"/>
+      <c r="M51" s="138"/>
+      <c r="N51" s="138"/>
+      <c r="O51" s="37">
+        <f>SUM(O3:O48)</f>
         <v>87.407999999999987</v>
       </c>
-      <c r="P51" s="38">
-        <f>P50/80</f>
+      <c r="Q51" s="38">
+        <f>Q50/80</f>
         <v>54.184811999999987</v>
       </c>
-    </row>
-    <row r="52" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R51" s="38"/>
+      <c r="S51" s="38">
+        <f>S50/110</f>
+        <v>49.258920000000018</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B52" s="36"/>
       <c r="C52" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="53" spans="1:17" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B53" s="36"/>
       <c r="C53" s="109" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="54" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C54" s="109"/>
     </row>
-    <row r="55" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C55" s="109"/>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C56" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="J50:N50"/>
+    <mergeCell ref="J51:N51"/>
+    <mergeCell ref="B27:B40"/>
     <mergeCell ref="B25:B26"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:T1"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="B3:B15"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="J50:M50"/>
-    <mergeCell ref="J51:M51"/>
-    <mergeCell ref="B27:B40"/>
   </mergeCells>
-  <conditionalFormatting sqref="N51:P51">
+  <conditionalFormatting sqref="O51:S51">
     <cfRule type="dataBar" priority="6">
       <dataBar>
         <cfvo type="min"/>
@@ -4708,7 +5288,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N23:N48 N3:N21">
+  <conditionalFormatting sqref="O23:O48 O3:O21">
     <cfRule type="dataBar" priority="19">
       <dataBar>
         <cfvo type="min"/>
@@ -4722,7 +5302,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P23:P48 P3:P21">
+  <conditionalFormatting sqref="Q23:Q48 Q3:Q21 S3:S48">
     <cfRule type="dataBar" priority="22">
       <dataBar>
         <cfvo type="min"/>
@@ -4736,7 +5316,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J3:K49">
+  <conditionalFormatting sqref="J3:L49">
     <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="min"/>
@@ -4750,52 +5330,52 @@
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="F9" tooltip="Manufacturer" display="'GCM1555C1H470JA16D"/>
-    <hyperlink ref="L4" r:id="rId1"/>
-    <hyperlink ref="L5" r:id="rId2"/>
-    <hyperlink ref="L6" r:id="rId3"/>
-    <hyperlink ref="L12" r:id="rId4"/>
-    <hyperlink ref="L14" r:id="rId5"/>
-    <hyperlink ref="L24" r:id="rId6"/>
-    <hyperlink ref="L26" r:id="rId7"/>
-    <hyperlink ref="L28" r:id="rId8"/>
-    <hyperlink ref="L29" r:id="rId9"/>
-    <hyperlink ref="L30" r:id="rId10"/>
-    <hyperlink ref="L31" r:id="rId11"/>
-    <hyperlink ref="L32" r:id="rId12"/>
-    <hyperlink ref="L33" r:id="rId13"/>
-    <hyperlink ref="L36" r:id="rId14"/>
-    <hyperlink ref="L37" r:id="rId15"/>
-    <hyperlink ref="L39" r:id="rId16"/>
-    <hyperlink ref="L40" r:id="rId17"/>
-    <hyperlink ref="L43" r:id="rId18"/>
-    <hyperlink ref="L46" r:id="rId19"/>
-    <hyperlink ref="L47" r:id="rId20"/>
-    <hyperlink ref="L48" r:id="rId21"/>
-    <hyperlink ref="L3" r:id="rId22"/>
-    <hyperlink ref="L7" r:id="rId23"/>
-    <hyperlink ref="L9" r:id="rId24"/>
-    <hyperlink ref="L10" r:id="rId25"/>
-    <hyperlink ref="L11" r:id="rId26"/>
-    <hyperlink ref="L13" r:id="rId27"/>
-    <hyperlink ref="L16" r:id="rId28"/>
-    <hyperlink ref="L19" r:id="rId29"/>
-    <hyperlink ref="L34" r:id="rId30"/>
-    <hyperlink ref="L35" r:id="rId31"/>
-    <hyperlink ref="L38" r:id="rId32"/>
-    <hyperlink ref="L42" r:id="rId33"/>
-    <hyperlink ref="L44" r:id="rId34"/>
-    <hyperlink ref="L41" r:id="rId35"/>
-    <hyperlink ref="L18" r:id="rId36"/>
-    <hyperlink ref="L22" r:id="rId37"/>
-    <hyperlink ref="L8" r:id="rId38"/>
-    <hyperlink ref="L15" r:id="rId39"/>
-    <hyperlink ref="L17" r:id="rId40"/>
-    <hyperlink ref="L20" r:id="rId41"/>
-    <hyperlink ref="L21" r:id="rId42"/>
-    <hyperlink ref="L23" r:id="rId43"/>
-    <hyperlink ref="L25" r:id="rId44"/>
-    <hyperlink ref="L27" r:id="rId45"/>
-    <hyperlink ref="L45" r:id="rId46"/>
+    <hyperlink ref="M4" r:id="rId1"/>
+    <hyperlink ref="M5" r:id="rId2"/>
+    <hyperlink ref="M6" r:id="rId3"/>
+    <hyperlink ref="M12" r:id="rId4"/>
+    <hyperlink ref="M14" r:id="rId5"/>
+    <hyperlink ref="M24" r:id="rId6"/>
+    <hyperlink ref="M26" r:id="rId7"/>
+    <hyperlink ref="M28" r:id="rId8"/>
+    <hyperlink ref="M29" r:id="rId9"/>
+    <hyperlink ref="M30" r:id="rId10"/>
+    <hyperlink ref="M31" r:id="rId11"/>
+    <hyperlink ref="M32" r:id="rId12"/>
+    <hyperlink ref="M33" r:id="rId13"/>
+    <hyperlink ref="M36" r:id="rId14"/>
+    <hyperlink ref="M37" r:id="rId15"/>
+    <hyperlink ref="M39" r:id="rId16"/>
+    <hyperlink ref="M40" r:id="rId17"/>
+    <hyperlink ref="M43" r:id="rId18"/>
+    <hyperlink ref="M46" r:id="rId19"/>
+    <hyperlink ref="M47" r:id="rId20"/>
+    <hyperlink ref="M48" r:id="rId21"/>
+    <hyperlink ref="M3" r:id="rId22"/>
+    <hyperlink ref="M7" r:id="rId23"/>
+    <hyperlink ref="M9" r:id="rId24"/>
+    <hyperlink ref="M10" r:id="rId25"/>
+    <hyperlink ref="M11" r:id="rId26"/>
+    <hyperlink ref="M13" r:id="rId27"/>
+    <hyperlink ref="M16" r:id="rId28"/>
+    <hyperlink ref="M19" r:id="rId29"/>
+    <hyperlink ref="M34" r:id="rId30"/>
+    <hyperlink ref="M35" r:id="rId31"/>
+    <hyperlink ref="M38" r:id="rId32"/>
+    <hyperlink ref="M42" r:id="rId33"/>
+    <hyperlink ref="M44" r:id="rId34"/>
+    <hyperlink ref="M41" r:id="rId35"/>
+    <hyperlink ref="M18" r:id="rId36"/>
+    <hyperlink ref="M22" r:id="rId37"/>
+    <hyperlink ref="M8" r:id="rId38"/>
+    <hyperlink ref="M15" r:id="rId39"/>
+    <hyperlink ref="M17" r:id="rId40"/>
+    <hyperlink ref="M20" r:id="rId41"/>
+    <hyperlink ref="M21" r:id="rId42"/>
+    <hyperlink ref="M23" r:id="rId43"/>
+    <hyperlink ref="M25" r:id="rId44"/>
+    <hyperlink ref="M27" r:id="rId45"/>
+    <hyperlink ref="M45" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId47"/>
@@ -4813,7 +5393,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>N51:P51</xm:sqref>
+          <xm:sqref>O51:S51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{BED3E9A7-7C6C-42CF-BFA0-C7FF39D6E667}">
@@ -4826,7 +5406,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>N23:N48 N3:N21</xm:sqref>
+          <xm:sqref>O23:O48 O3:O21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{15F47113-5465-446D-AE26-CA793756D32B}">
@@ -4839,7 +5419,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P23:P48 P3:P21</xm:sqref>
+          <xm:sqref>Q23:Q48 Q3:Q21 S3:S48</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>